<commit_message>
ACDR2026: agenda 0930 (COJ, Joint Opening order, no co-moderator); opening remarks rev3 (3 min); scenario timings; drafts to Kodama and Yoshida
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_0930_rev2.xlsx
+++ b/reports/acdr2026_staff_deployment/進行シナリオ_0929/ACDR2026_進行シナリオ_Opening_RT_TS_CS_0930_rev2.xlsx
@@ -549,7 +549,8 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催、APMCDRR と back-to-back、2027年10月（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
+          <t>・RT: Co-Moderator は置かない（Gerry・吉田 9/30）。
+・Closing: Summary＝宮木所長（Gerry 起草）、Closing Remarks＝三浦センター長（Chairman）＋SCDF側【SCDF 登壇者は Sylvia と要確認】。次回 ACDR は仙台開催、APMCDRR と back-to-back、2027年10月（閉会挨拶で発表）。10月時点の肩書: 所長＝Executive Director（11/1 以降は北本氏が ED、宮木氏が Director General）。次回開催地の発表有無も未定。</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1221,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Opening Remarks (3) Government of Japan</t>
+          <t>Opening Remarks (3) Cabinet Office of Japan (COJ)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -1230,7 +1231,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Lastly, I am pleased to invite Mr HAYASHI Masamichi, Deputy Minister, Government of Japan, to deliver his opening remarks. Deputy Minister Hayashi, please.
+          <t>Lastly, I am pleased to invite Mr HAYASHI Masamichi, Deputy Minister, Cabinet Office of Japan (COJ), to deliver his opening remarks. Deputy Minister Hayashi, please.
 （挨拶 約4分）
 Thank you very much, Deputy Minister Hayashi.</t>
         </is>
@@ -1352,7 +1353,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Moderator: SCDF（LTC Chen Yong Kai）。Co-Moderator: ADRC メンバー国【TBC】。ADRC 運営: 吉田（PIC・進行補助・ベル）、Gerry（ノート・サマリー）、池田（PC・スクリーン）、荒木田（AV/Zoom）。</t>
+          <t>Moderator: SCDF（LTC Chen Yong Kai）単独（Co-Moderator は置かない: Gerry・吉田 9/30 合意、2025 も喜多参事官単独）。ADRC 運営: 吉田（PIC・進行補助・ベル）、Gerry（ノート・サマリー）、池田（PC・スクリーン）、荒木田（AV/Zoom）。</t>
         </is>
       </c>
       <c r="G16" s="6" t="n"/>
@@ -1391,7 +1392,7 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Co-Moderator を置く場合はここで紹介し、後半（国際機関）の進行を任せる案。ベルは吉田。Q&amp;A方式【TBC】。</t>
+          <t>Co-Moderator なし（9/30 決定）。ベルは吉田。Q&amp;A方式は吉田・Gerry 回答待ち。</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -4686,24 +4687,24 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Presentation 6: Japan (Cabinet Office)</t>
+          <t>Presentation 6: Cabinet Office of Japan (COJ)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>PPT 17-6: Name（Japan (Cabinet Office)）→ 発表スライド</t>
+          <t>PPT 17-6: Name（Cabinet Office of Japan (COJ)）→ 発表スライド</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Our sixth presentation is from Japan (Cabinet Office). May I invite Cabinet Office, Government of Japan: 1-minute introduction + Spectee + one more company. Please.
+          <t>Our sixth presentation is from Cabinet Office of Japan (COJ). May I invite Cabinet Office of Japan (COJ): 1-minute introduction + Spectee + WOTA（計15分。児玉 9/30: 発表者は Spectee 根来氏・WOTA 郷坪氏の見込み、確認中）. Please.
 （発表 15分）
 Thank you very much.</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Cabinet Office, Government of Japan: 1-minute introduction + Spectee + one more company【TBC】（計15分）
+          <t>Cabinet Office of Japan (COJ): 1-minute introduction + Spectee + WOTA（計15分。児玉 9/30: 発表者は Spectee 根来氏・WOTA 郷坪氏の見込み、確認中）
 内閣府枠は中根氏が1分イントロ。前方席8席の入替なし。</t>
         </is>
       </c>
@@ -5365,7 +5366,7 @@
           <t>Opening Remarks (order per SCDF, tbc):
 – Prof. MIURA Fusanori, Chairman, Asian Disaster Reduction Center
 – Mr Eric Yap Wee Teck, Commissioner, Singapore Civil Defence Force (tbc)
-– Mr HAYASHI Masamichi, Deputy Minister, Government of Japan
+– Mr HAYASHI Masamichi, Deputy Minister, Cabinet Office of Japan (COJ)
 Emcee: LTC Chen Yong Kai, SCDF</t>
         </is>
       </c>
@@ -5421,7 +5422,7 @@
       <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Roundtable Session: Progress and Remaining Challenges in Implementing SFDRR 2015-2030
-Moderator: Singapore Civil Defence Force / Co-Moderator: [ADRC member country]</t>
+Moderator: Singapore Civil Defence Force</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -5629,7 +5630,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>6枠: Google (Ms Sirada Boonkongchuen) / JAXA / BRIN (Dr Yenni Vetrita) / YI-Lab (Mr Pradip Khatiwada) / Uzbekistan / Cabinet Office of Japan (Spectee + 1)</t>
+          <t>6枠: Google (Ms Sirada Boonkongchuen) / JAXA / BRIN (Dr Yenni Vetrita) / YI-Lab (Mr Pradip Khatiwada) / Uzbekistan / Cabinet Office of Japan (COJ: Spectee + WOTA)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">

</xml_diff>